<commit_message>
Modifications as per CRA internal review
</commit_message>
<xml_diff>
--- a/statvar_imports/database_on_indian_economy/india_rbi_state_statistics/testdata/environment_input.xlsx
+++ b/statvar_imports/database_on_indian_economy/india_rbi_state_statistics/testdata/environment_input.xlsx
@@ -1,14 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="T_99(i)" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="T_99(ii)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T_99(i)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T_99(ii)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T_102(i)" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -604,7 +605,6 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
           <t>State/Union Territory</t>
@@ -3121,7 +3121,6 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
           <t>State/Union Territory</t>
@@ -5717,6 +5716,160 @@
       <c r="K49" t="inlineStr">
         <is>
           <t>nan</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1"/>
+    <row r="2">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>TABLE 102: SUB-DIVISION-WISE ANNUAL RAINFALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>(Millimeter)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>State/Union Territory</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D4" t="n">
+        <v>2001</v>
+      </c>
+      <c r="E4" t="n">
+        <v>2002</v>
+      </c>
+      <c r="F4" t="n">
+        <v>2003</v>
+      </c>
+      <c r="G4" t="n">
+        <v>2004</v>
+      </c>
+      <c r="H4" t="n">
+        <v>2005</v>
+      </c>
+      <c r="I4" t="n">
+        <v>2006</v>
+      </c>
+      <c r="J4" t="n">
+        <v>2007</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Andaman &amp; Nicobar Islands</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2763.2</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>3080.9</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2620.2</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2355.9</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2460.1</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2954.7</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>2404.7</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>2748.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Haryana, Delhi &amp; Chandigarh</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>384.4</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>485.5</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>357.2</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>597.6</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>487.3</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>519.5</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>330.9</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>446.6</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
[India_RBI_State_Statistics] Modified download script and handle deletions (#2201)
* Modified download script and handle deletions

* Made changes suggested by Gemini-bot

* Changes as per recommendation

* Changes made as per comments

* Made changes in downlaod script

* Modified naming in config.json

* Resolved comments

* CRA analysis done

* Changes as per Internal reviews

* CRA based changes

* Modified changes as per Internal CRA report

* Modifications as per CRA internal review

* Changed run.sh first line

* Modified readme.md to set 0.1%

* Modifications as per review comments

* Changes made as per comments

* Changes made to resolve comments

* Clean up the manifest.json

* Cleaning up manifest and download script

* Modified readme.md and pvmap

* Fix rbi_download.py merge resolution and format with yapf
</commit_message>
<xml_diff>
--- a/statvar_imports/database_on_indian_economy/india_rbi_state_statistics/testdata/environment_input.xlsx
+++ b/statvar_imports/database_on_indian_economy/india_rbi_state_statistics/testdata/environment_input.xlsx
@@ -1,14 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="T_99(i)" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="T_99(ii)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T_99(i)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T_99(ii)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T_102(i)" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -604,7 +605,6 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
           <t>State/Union Territory</t>
@@ -3121,7 +3121,6 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
           <t>State/Union Territory</t>
@@ -5717,6 +5716,160 @@
       <c r="K49" t="inlineStr">
         <is>
           <t>nan</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1"/>
+    <row r="2">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>TABLE 102: SUB-DIVISION-WISE ANNUAL RAINFALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>(Millimeter)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>State/Union Territory</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D4" t="n">
+        <v>2001</v>
+      </c>
+      <c r="E4" t="n">
+        <v>2002</v>
+      </c>
+      <c r="F4" t="n">
+        <v>2003</v>
+      </c>
+      <c r="G4" t="n">
+        <v>2004</v>
+      </c>
+      <c r="H4" t="n">
+        <v>2005</v>
+      </c>
+      <c r="I4" t="n">
+        <v>2006</v>
+      </c>
+      <c r="J4" t="n">
+        <v>2007</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Andaman &amp; Nicobar Islands</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2763.2</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>3080.9</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2620.2</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2355.9</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2460.1</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2954.7</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>2404.7</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>2748.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Haryana, Delhi &amp; Chandigarh</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>384.4</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>485.5</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>357.2</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>597.6</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>487.3</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>519.5</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>330.9</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>446.6</t>
         </is>
       </c>
     </row>

</xml_diff>